<commit_message>
Add BCV USD historical exchange rate pipeline
</commit_message>
<xml_diff>
--- a/assets/data/bcv/excel/ove_bcv_tipo_cambio_referencia_smc.xlsx
+++ b/assets/data/bcv/excel/ove_bcv_tipo_cambio_referencia_smc.xlsx
@@ -7,56 +7,131 @@
 </workbook>
 </file>
 
+<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <fonts count="2">
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0B1D3D"/>
+      <name val="Inter"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Inter"/>
+    </font>
+  </fonts>
+  <fills count="3">
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF0A2D5A"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+  </fills>
+  <borders count="1">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+  </borders>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+  </cellStyleXfs>
+  <cellXfs count="2">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+  </cellXfs>
+  <cellStyles count="1">
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+  </cellStyles>
+</styleSheet>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <cols>
+    <col min="1" max="1" width="28" customWidth="1"/>
+    <col min="2" max="2" width="28" customWidth="1"/>
+    <col min="3" max="3" width="18" customWidth="1"/>
+    <col min="4" max="4" width="18" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="18" customWidth="1"/>
+    <col min="7" max="7" width="18" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="18" customWidth="1"/>
+    <col min="10" max="10" width="18" customWidth="1"/>
+    <col min="11" max="11" width="18" customWidth="1"/>
+    <col min="12" max="12" width="18" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>indicator_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>indicator_name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>date</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>value</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>value_buy</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>value_sell</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>frequency</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>source_url</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>fetched_at</t>
         </is>
@@ -83,32 +158,42 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
           <t>CNY</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="H2" t="inlineStr">
         <is>
           <t>VES por unidad de moneda extranjera</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>daily</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>Banco Central de Venezuela</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>2026-06-26T09:35:29Z</t>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:47:00Z</t>
         </is>
       </c>
     </row>
@@ -133,32 +218,42 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
           <t>EUR</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>VES por unidad de moneda extranjera</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>daily</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>Banco Central de Venezuela</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>2026-06-26T09:35:29Z</t>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:47:00Z</t>
         </is>
       </c>
     </row>
@@ -183,32 +278,42 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
           <t>RUB</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>VES por unidad de moneda extranjera</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>daily</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>Banco Central de Venezuela</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>2026-06-26T09:35:29Z</t>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:47:00Z</t>
         </is>
       </c>
     </row>
@@ -233,32 +338,42 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
           <t>TRY</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>VES por unidad de moneda extranjera</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>daily</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Banco Central de Venezuela</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>2026-06-26T09:35:29Z</t>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:47:00Z</t>
         </is>
       </c>
     </row>
@@ -283,32 +398,42 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
           <t>USD</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>VES por unidad de moneda extranjera</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>daily</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>Banco Central de Venezuela</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>2026-06-26T09:35:29Z</t>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-06-26T17:47:00Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update Venezuela data sources
</commit_message>
<xml_diff>
--- a/assets/data/bcv/excel/ove_bcv_tipo_cambio_referencia_smc.xlsx
+++ b/assets/data/bcv/excel/ove_bcv_tipo_cambio_referencia_smc.xlsx
@@ -437,6 +437,306 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_cny</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - CNY</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>100.9793608</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-07-07T22:56:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_eur</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - EUR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D8">
+        <v>783.7787073</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-07-07T22:56:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_rub</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - RUB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>8.97360936</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-07-07T22:56:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_try</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - TRY</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>14.64594213</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>TRY</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-07-07T22:56:56Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_usd</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - USD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D11">
+        <v>685.9427</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-07-07T22:56:56Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update Venezuela observatory data
</commit_message>
<xml_diff>
--- a/assets/data/bcv/excel/ove_bcv_tipo_cambio_referencia_smc.xlsx
+++ b/assets/data/bcv/excel/ove_bcv_tipo_cambio_referencia_smc.xlsx
@@ -437,6 +437,306 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_cny</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - CNY</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D7">
+        <v>100.9793608</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>CNY</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-07-08T07:42:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_eur</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - EUR</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D8">
+        <v>783.7787073</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2026-07-08T07:42:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_rub</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - RUB</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D9">
+        <v>8.97360936</v>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>RUB</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>2026-07-08T07:42:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_try</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - TRY</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D10">
+        <v>14.64594213</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>TRY</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>2026-07-08T07:42:32Z</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>bcv_tipo_cambio_referencia_smc_usd</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tipo de Cambio de Referencia SMC - USD</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="D11">
+        <v>685.9427</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>VES por unidad de moneda extranjera</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>daily</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Banco Central de Venezuela</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>https://www.bcv.org.ve/estadisticas/tipo-cambio-de-referencia-smc</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>2026-07-08T07:42:32Z</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>